<commit_message>
Docs: ERS-01 v1.3, CU-01 v2.4 e HU-17 con la API de materiales - Camila Olivares
Caso CU-REP-08, diagrama del paquete 10 y avance del Sprint 3 al 22-10.
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/2. Metodología Scrum/SPRINTS/SITRAFO_Product_Backlog.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/2. Metodología Scrum/SPRINTS/SITRAFO_Product_Backlog.xlsx
@@ -1206,7 +1206,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Planificada</t>
+          <t xml:space="preserve">En curso</t>
         </is>
       </c>
       <c r="F21" s="5" t="n">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>HU-17 en la ERS-01 (RF-INV-09). Historia y criterios: Camila Olivares (20-oct); desarrollo: Benjamín Delgado (21 y 22-oct); pruebas: Milko Soto (23-oct).</t>
+          <t xml:space="preserve">HU-17 en la ERS-01 (RF-INV-09) y CU-REP-08 en el CU-01. Historia y criterios: Camila Olivares (19-oct, ajustados el 22-oct); desarrollo: Benjamín Delgado (21-oct, en el repositorio el 22-oct, con 12 pruebas automatizadas); pruebas manuales: Milko Soto (pendiente).</t>
         </is>
       </c>
     </row>

</xml_diff>